<commit_message>
Rename vulnerability seed workbook to 1-Codes-basing
</commit_message>
<xml_diff>
--- a/HLT-vkl-26/backend/database/seed_sources/1-Codes-basing.xlsx
+++ b/HLT-vkl-26/backend/database/seed_sources/1-Codes-basing.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931B4B3D-D6F6-438D-A210-42A690237A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1193E1-3B34-451B-9E2A-1CD8237D9556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1290" yWindow="3075" windowWidth="21600" windowHeight="11400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
   <si>
     <t>snmp-info</t>
   </si>
@@ -98,27 +98,12 @@
     <t>Cập nhật phpMyAdmin lên phiên bản 4.x+, tắt hoặc giới hạn truy cập phpMyAdmin</t>
   </si>
   <si>
-    <t>CVE-2011-3192: dịch vụ Apache HTTP Server phiên bản cũ, có thể bị tấn công DoS qua Range header với nhiều dải chồng lấn.</t>
-  </si>
-  <si>
-    <t>Nâng cấp Apache HTTP Server lên bản 2.2.21 hoặc 2.4 trở lên, cấu hình hạn chế hoặc loại bỏ Range header.</t>
-  </si>
-  <si>
-    <t>CVE-2013-0156: Ứng dụng Ruby on Rails phiên bản cũ cho phép attacker thực hiện object injection thông qua xử lý tham số không an toàn, dẫn đến nguy cơ thực thi mã từ xa hoặc gây từ chối dịch vụ.</t>
-  </si>
-  <si>
-    <t>Nâng cấp Ruby on Rails lên phiên bản 3.2.11+ và vô hiệu hóa xử lý YAML/XML không cần thiết trong truyền tham số.</t>
-  </si>
-  <si>
     <t>CVE-2014-0224: HTTPS sử dụng thư viện TLS chưa cập nhật bản vá, attacker có thể từ vị trì MITM chèn gói ChangeCipherSpec giả, làm vô hiệu hóa mã hóa TLS</t>
   </si>
   <si>
     <t>Cập nhật thư viện TLS (Open SSL 1.0.1h+)</t>
   </si>
   <si>
-    <t>CVE-2014-3566: POODLE, attacker có thể từ vị trí MITM ép downgrade từ TLS sang SSLv3 trong Schannel.</t>
-  </si>
-  <si>
     <t>Tắt SSLv3 trong Schannel, bật và ưu tiên TLS 1.0/1.1/1.2, tắt SSDP/UOPnP nếu không dùng</t>
   </si>
   <si>
@@ -131,15 +116,9 @@
     <t>http-cross-domain-policy: Cấu hình file cross-domain rộng, có thể cho phép domain không tin cậy truy cập tài nguyên hoặc API của hệ thống</t>
   </si>
   <si>
-    <t>Rà soát và giới hạn file crossdomain.xml hoặc clientaccesspolicy.xml, chỉ cho phép các domain tin cậy, hoặc gỡ bỏ nếu không còn sử dụng Flash/Silverlight.</t>
-  </si>
-  <si>
     <t>http-method-tamper: dịch vụ http cho phép các method không cần thiết, có thể bị lợi dụng để bypass kiểm soát truy cập, thay đổi dữ liệu hoặc thu thập thông tin hệ thống</t>
   </si>
   <si>
-    <t>Rà soát dịch vụ web, chỉ cho phép các method cần thiết, tắt hoặc vô hiệu hóa các method không sử dụng.</t>
-  </si>
-  <si>
     <t>http-vuln-cve2010-0738: dịch vụ Jboss Application Server cũ, chỉ kiểm tra quyền với HTTP GET mà không kiểm tra đầy đủ với POST, dẫn đến khả năng truy cập trái phép vào giao diện quản trị JMX Console</t>
   </si>
   <si>
@@ -149,15 +128,9 @@
     <t>http-vuln-cve2015-1635: hệ điều hành Windows cũ, tồn tại lỗ hổng CVE-2015-1635 trong thành phần HTTP.sys cho phép attacker thực thi mã từ xa với quyền System thông qua các request HTTP được sửa đổi</t>
   </si>
   <si>
-    <t>http-vuln-cve2017-1001000: dịch vụ Wordpress cũ, tồn tại lỗ hổng REST API cho phép chỉnh sửa nội dung bài viết mà không cần xác thực.</t>
-  </si>
-  <si>
     <t>Cập nhật Wordpress lên bản 4.7.2 trở lên.</t>
   </si>
   <si>
-    <t>snmp-info: có nguy cơ lộ lọt thông tin snmp</t>
-  </si>
-  <si>
     <t>Tắt hoặc chuyển sang SNMPv3</t>
   </si>
   <si>
@@ -167,34 +140,49 @@
     <t>Để thực hiện tấn công phải ở cùng mạng với nạn nhân (để thực hiện MiTM) nên không tiến hành chứng minh.</t>
   </si>
   <si>
-    <t>CVE-2005-3299: Đang xác minh.</t>
-  </si>
-  <si>
-    <t>CVE-2013-0156: Đang xác minh.</t>
-  </si>
-  <si>
-    <t>CVE-2015-1635: Đang xác minh.</t>
-  </si>
-  <si>
-    <t>http-cross-domain-policy: Đang xác minh.</t>
-  </si>
-  <si>
-    <t>http-method-tamper: Đang xác minh.</t>
-  </si>
-  <si>
-    <t>http-vuln-cve2010-0738: Đang xác minh.</t>
-  </si>
-  <si>
-    <t>http-vuln-cve2015-1635: Đang xác minh.</t>
-  </si>
-  <si>
-    <t>http-vuln-cve2017-1001000: Đang xác minh.</t>
-  </si>
-  <si>
     <t>CVE-2011-3192: Lỗ hổng liên quan DoS nên không tiến hành chứng minh.</t>
   </si>
   <si>
     <t>snmp-info-poc.py</t>
+  </si>
+  <si>
+    <t>http-frontpage-login</t>
+  </si>
+  <si>
+    <t>http-frontpage-login: tồn tại cấu hình Microsoft Frontpage Extensions cũ, có nguy cơ cho phép đăng nhập ẩn danh vào hệ thống, từ đó có thể chỉnh sửa nội dung, tải tệp độc hại, chiếm quyền điều khiển máy chủ web</t>
+  </si>
+  <si>
+    <t>http-vuln-cve2017-1001000: dịch vụ Wordpress cũ, tồn tại lỗ hổng REST API cho phép chỉnh sửa nội dung bài viết mà không cần xác thực</t>
+  </si>
+  <si>
+    <t>CVE-2014-3566: POODLE, attacker có thể từ vị trí MITM ép downgrade từ TLS sang SSLv3 trong Schannel</t>
+  </si>
+  <si>
+    <t>CVE-2013-0156: Ứng dụng Ruby on Rails phiên bản cũ cho phép attacker thực hiện object injection thông qua xử lý tham số không an toàn, dẫn đến nguy cơ thực thi mã từ xa hoặc gây từ chối dịch vụ</t>
+  </si>
+  <si>
+    <t>CVE-2011-3192: dịch vụ Apache HTTP Server phiên bản cũ, có thể bị tấn công DoS qua Range header với nhiều dải chồng lấn</t>
+  </si>
+  <si>
+    <t>Nâng cấp Apache HTTP Server lên bản 2.2.21 hoặc 2.4 trở lên, cấu hình hạn chế hoặc loại bỏ Range header</t>
+  </si>
+  <si>
+    <t>Nâng cấp Ruby on Rails lên phiên bản 3.2.11+ và vô hiệu hóa xử lý YAML/XML không cần thiết trong truyền tham số</t>
+  </si>
+  <si>
+    <t>Cập nhật bản vá bảo mật MS15-034 hoặc tương đương (KB3033929) cho hệ điều hành</t>
+  </si>
+  <si>
+    <t>Rà soát và giới hạn file crossdomain.xml hoặc clientaccesspolicy.xml, chỉ cho phép các domain tin cậy, hoặc gỡ bỏ nếu không còn sử dụng Flash/Silverlight</t>
+  </si>
+  <si>
+    <t>Rà soát dịch vụ web, chỉ cho phép các method cần thiết, tắt hoặc vô hiệu hóa các method không sử dụng</t>
+  </si>
+  <si>
+    <t>Kiểm tra và vô hiệu hóa toàn bộ FrontPage Extensions hoặc các thành phần _vti_* không con sử dụng, đồng thời cập nhật cấu hình xác thực và giới hạn truy cập quản trị</t>
+  </si>
+  <si>
+    <t>snmp-info: lộ thông tin về tên thiết bị, phiên bản phần mềm cụ thể, địa chỉ IP, cấu hình định tuyến và một số thông tin khác</t>
   </si>
 </sst>
 </file>
@@ -562,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -582,7 +570,7 @@
         <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>15</v>
@@ -598,9 +586,7 @@
       <c r="C2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>48</v>
-      </c>
+      <c r="D2" s="3"/>
       <c r="E2" s="4">
         <v>3</v>
       </c>
@@ -610,13 +596,13 @@
         <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="E3" s="4">
         <v>3</v>
@@ -627,14 +613,12 @@
         <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>49</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="D4" s="3"/>
       <c r="E4" s="4">
         <v>4</v>
       </c>
@@ -644,13 +628,13 @@
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E5" s="4">
         <v>2</v>
@@ -661,13 +645,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E6" s="4">
         <v>2</v>
@@ -678,14 +662,12 @@
         <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>50</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="D7" s="3"/>
       <c r="E7" s="4">
         <v>4</v>
       </c>
@@ -695,14 +677,12 @@
         <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>51</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="D8" s="3"/>
       <c r="E8" s="4">
         <v>2</v>
       </c>
@@ -712,14 +692,12 @@
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>52</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="D9" s="3"/>
       <c r="E9" s="4">
         <v>2</v>
       </c>
@@ -729,14 +707,12 @@
         <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>53</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="D10" s="3"/>
       <c r="E10" s="4">
         <v>3</v>
       </c>
@@ -746,14 +722,12 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>54</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="D11" s="3"/>
       <c r="E11" s="4">
         <v>4</v>
       </c>
@@ -763,32 +737,45 @@
         <v>3</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>55</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="D12" s="3"/>
       <c r="E12" s="4">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E13" s="4">
+      <c r="B14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="4">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-create unknown CVE records from scan results and relabel level zero
</commit_message>
<xml_diff>
--- a/HLT-vkl-26/backend/database/seed_sources/1-Codes-basing.xlsx
+++ b/HLT-vkl-26/backend/database/seed_sources/1-Codes-basing.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1193E1-3B34-451B-9E2A-1CD8237D9556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD74E42B-06A8-45CA-91C2-2D6C75E78689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="53">
   <si>
     <t>snmp-info</t>
   </si>
@@ -77,9 +77,6 @@
     <t>Text</t>
   </si>
   <si>
-    <t>Thông tin</t>
-  </si>
-  <si>
     <t>Thấp</t>
   </si>
   <si>
@@ -110,9 +107,6 @@
     <t>CVE-2015-1635: hệ điều hành Windows cũ, tồn tại lỗ hổng CVE-2015-1635 trong thành phần HTTP.sys cho phép attacker thực thi mã từ xa với quyền System thông qua các request HTTP được sửa đổi</t>
   </si>
   <si>
-    <t>Cập nhật bản vá bảo mật MS15-034 hoặc tương đương (KB3033929) cho hệ điều hành.</t>
-  </si>
-  <si>
     <t>http-cross-domain-policy: Cấu hình file cross-domain rộng, có thể cho phép domain không tin cậy truy cập tài nguyên hoặc API của hệ thống</t>
   </si>
   <si>
@@ -122,27 +116,15 @@
     <t>http-vuln-cve2010-0738: dịch vụ Jboss Application Server cũ, chỉ kiểm tra quyền với HTTP GET mà không kiểm tra đầy đủ với POST, dẫn đến khả năng truy cập trái phép vào giao diện quản trị JMX Console</t>
   </si>
   <si>
-    <t>Cập nhật Jboss EAP/JBossAS lên bản 4.2.0.CP09 hoặc 4.3.0.CP08 trở lên.</t>
-  </si>
-  <si>
     <t>http-vuln-cve2015-1635: hệ điều hành Windows cũ, tồn tại lỗ hổng CVE-2015-1635 trong thành phần HTTP.sys cho phép attacker thực thi mã từ xa với quyền System thông qua các request HTTP được sửa đổi</t>
   </si>
   <si>
-    <t>Cập nhật Wordpress lên bản 4.7.2 trở lên.</t>
-  </si>
-  <si>
     <t>Tắt hoặc chuyển sang SNMPv3</t>
   </si>
   <si>
     <t>Kiểm chứng</t>
   </si>
   <si>
-    <t>Để thực hiện tấn công phải ở cùng mạng với nạn nhân (để thực hiện MiTM) nên không tiến hành chứng minh.</t>
-  </si>
-  <si>
-    <t>CVE-2011-3192: Lỗ hổng liên quan DoS nên không tiến hành chứng minh.</t>
-  </si>
-  <si>
     <t>snmp-info-poc.py</t>
   </si>
   <si>
@@ -183,6 +165,21 @@
   </si>
   <si>
     <t>snmp-info: lộ thông tin về tên thiết bị, phiên bản phần mềm cụ thể, địa chỉ IP, cấu hình định tuyến và một số thông tin khác</t>
+  </si>
+  <si>
+    <t>Cập nhật Wordpress lên bản 4.7.2 trở lên</t>
+  </si>
+  <si>
+    <t>Cập nhật Jboss EAP/JBossAS lên bản 4.2.0.CP09 hoặc 4.3.0.CP08 trở lên</t>
+  </si>
+  <si>
+    <t>CVE-2011-3192: Lỗ hổng liên quan DoS nên không tiến hành chứng minh</t>
+  </si>
+  <si>
+    <t>Để thực hiện tấn công phải ở cùng mạng với nạn nhân (để thực hiện MiTM) nên không tiến hành chứng minh</t>
+  </si>
+  <si>
+    <t>Chưa xác định</t>
   </si>
 </sst>
 </file>
@@ -570,7 +567,7 @@
         <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>15</v>
@@ -581,10 +578,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="4">
@@ -596,13 +593,13 @@
         <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E3" s="4">
         <v>3</v>
@@ -613,10 +610,10 @@
         <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="4">
@@ -628,13 +625,13 @@
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>26</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="E5" s="4">
         <v>2</v>
@@ -645,13 +642,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="E6" s="4">
         <v>2</v>
@@ -662,10 +659,10 @@
         <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="4">
@@ -677,10 +674,10 @@
         <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="4">
@@ -692,10 +689,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="4">
@@ -707,10 +704,10 @@
         <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="4">
@@ -722,10 +719,10 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="4">
@@ -737,10 +734,10 @@
         <v>3</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="4">
@@ -749,13 +746,13 @@
     </row>
     <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="4">
@@ -767,16 +764,16 @@
         <v>0</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="E14" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -809,7 +806,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -817,7 +814,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -825,7 +822,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -833,7 +830,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -841,7 +838,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Upgrade agent monitoring runtime and redesign agents dashboard
</commit_message>
<xml_diff>
--- a/HLT-vkl-26/backend/database/seed_sources/1-Codes-basing.xlsx
+++ b/HLT-vkl-26/backend/database/seed_sources/1-Codes-basing.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD74E42B-06A8-45CA-91C2-2D6C75E78689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{411ECDE6-5CDD-4793-9739-8DBD9B6FD833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="2" r:id="rId1"/>

</xml_diff>